<commit_message>
fix(examples): limit the park control output of the IECB2020 performance examples so it does not wind up during the dip
</commit_message>
<xml_diff>
--- a/examples/Performance/Single/IECB2020/Excel/Producer.xlsx
+++ b/examples/Performance/Single/IECB2020/Excel/Producer.xlsx
@@ -13176,7 +13176,7 @@
         <v>359</v>
       </c>
       <c r="N10" s="101">
-        <v>999</v>
+        <v>0.5</v>
       </c>
       <c r="O10" s="98" t="s">
         <v>330</v>
@@ -13224,7 +13224,7 @@
         <v>364</v>
       </c>
       <c r="N11" s="101">
-        <v>-999</v>
+        <v>-0.5</v>
       </c>
       <c r="O11" s="98" t="s">
         <v>330</v>
@@ -13368,7 +13368,7 @@
         <v>377</v>
       </c>
       <c r="N14" s="101">
-        <v>999</v>
+        <v>0.5</v>
       </c>
       <c r="O14" s="98" t="s">
         <v>330</v>
@@ -13416,7 +13416,7 @@
         <v>381</v>
       </c>
       <c r="N15" s="101">
-        <v>-999</v>
+        <v>-0.5</v>
       </c>
       <c r="O15" s="98" t="s">
         <v>330</v>

</xml_diff>